<commit_message>
Kit La Foi : EAN 9782919843275
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lafoi_kit/fiche-technique-matrice.xlsx
+++ b/lafoi_kit/fiche-technique-matrice.xlsx
@@ -1246,7 +1246,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AX404"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="29.140625" customWidth="1" style="23" min="1" max="1"/>
     <col width="22.7109375" customWidth="1" style="23" min="2" max="2"/>
@@ -1554,7 +1554,11 @@
           <t>La Foi et ses piliers</t>
         </is>
       </c>
-      <c r="C2" s="109" t="n"/>
+      <c r="C2" s="110" t="inlineStr">
+        <is>
+          <t>9782919843275</t>
+        </is>
+      </c>
       <c r="D2" s="91" t="inlineStr">
         <is>
           <t>Un ouvrage pour initier les enfants aux piliers de la foi (imane) et de la croyance ('aqida) en islam. Plus de vingt thèmes entièrement illustrés et commentés, chacun mêlant un texte pédagogique, des illustrations et une bande dessinée, et accompagné d'extraits de versets du Coran ou de hadiths. Parmi les sujets traités : les signes qu'Allah existe, la croyance aux anges, aux livres révélés, au Paradis et à l'Enfer, au destin, au Jugement dernier.
@@ -4139,7 +4143,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
@@ -4181,17 +4185,17 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="101" t="inlineStr">
         <is>
-          <t>EAN</t>
+          <t>EAN · fait</t>
         </is>
       </c>
       <c r="B5" s="37" t="inlineStr">
         <is>
-          <t>Aucun EAN attribué au 23/09/2026 : le titre n’est pas encore dans la feuille « isbn BDOUIN ».</t>
+          <t>9782919843275, attribué par Karim le 23/09/2026.</t>
         </is>
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
-          <t>Karim, à attribuer</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4372,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:W42"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="23.7109375" customWidth="1" style="27" min="1" max="1"/>
     <col width="57.85546875" customWidth="1" style="88" min="2" max="2"/>
@@ -5111,7 +5115,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L1364"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="38" min="1" max="1"/>
     <col width="62.42578125" customWidth="1" min="12" max="12"/>
@@ -24453,7 +24457,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:XFD20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="24.28515625" customWidth="1" style="76" min="1" max="1"/>
     <col width="12.28515625" customWidth="1" style="26" min="2" max="2"/>

</xml_diff>